<commit_message>
Building and transportation calibration corrections
</commit_message>
<xml_diff>
--- a/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
+++ b/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmahajan\Documents\eps-us\InputData\trans\SoCDTtiNTY\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\trans\SoCDTtiNTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73732797-F0D5-4552-9011-A59D9397727A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24120B86-5063-4049-AFE6-30BB6A35CEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="960" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -117,6 +117,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="169" formatCode="0.000"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -154,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -166,6 +169,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -184,9 +188,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -224,9 +228,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -259,26 +263,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -311,26 +298,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -505,14 +475,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -520,47 +490,47 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -576,13 +546,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.08984375" customWidth="1"/>
-    <col min="2" max="8" width="14.36328125" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="2" max="8" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -608,33 +578,40 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="C2">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="D2">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="E2">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="F2">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="G2">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="H2">
-        <v>8.5999999999999993E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="B2" s="5">
+        <f>1/13</f>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="C2" s="5">
+        <f t="shared" ref="C2:H2" si="0">1/13</f>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="D2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="E2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="F2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="G2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+      <c r="H2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.6923076923076927E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -660,7 +637,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -686,7 +663,7 @@
         <v>4.1599999999999998E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -712,7 +689,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -738,7 +715,7 @@
         <v>2.9819999999999999E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -775,13 +752,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.08984375" customWidth="1"/>
-    <col min="2" max="8" width="14.36328125" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="2" max="8" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -807,7 +784,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -833,7 +810,7 @@
         <v>7.1999999999999995E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -859,7 +836,7 @@
         <v>3.5499999999999997E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -885,7 +862,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -911,7 +888,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -937,7 +914,7 @@
         <v>3.0300000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>17</v>
       </c>

</xml_diff>

<commit_message>
Correcting to include covid impacts, transportation calibration
</commit_message>
<xml_diff>
--- a/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
+++ b/InputData/trans/SoCDTtiNTY/Share of Cargo Dist Transported that is New This Year.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mary Francis Swint\Vensim\eps-indonesia\InputData\trans\SoCDTtiNTY\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24120B86-5063-4049-AFE6-30BB6A35CEEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D89E7B77-352E-424A-9482-9625A4C994E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="960" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32670" yWindow="-90" windowWidth="13620" windowHeight="11205" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -118,7 +118,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -169,7 +169,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -475,14 +475,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -490,47 +490,47 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -546,13 +546,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="8" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="2" max="8" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -578,66 +578,73 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="5">
-        <f>1/13</f>
-        <v>7.6923076923076927E-2</v>
+        <f>1/14</f>
+        <v>7.1428571428571425E-2</v>
       </c>
       <c r="C2" s="5">
-        <f t="shared" ref="C2:H2" si="0">1/13</f>
-        <v>7.6923076923076927E-2</v>
+        <f t="shared" ref="C2:H2" si="0">1/14</f>
+        <v>7.1428571428571425E-2</v>
       </c>
       <c r="D2" s="5">
         <f t="shared" si="0"/>
-        <v>7.6923076923076927E-2</v>
+        <v>7.1428571428571425E-2</v>
       </c>
       <c r="E2" s="5">
         <f t="shared" si="0"/>
-        <v>7.6923076923076927E-2</v>
+        <v>7.1428571428571425E-2</v>
       </c>
       <c r="F2" s="5">
         <f t="shared" si="0"/>
-        <v>7.6923076923076927E-2</v>
+        <v>7.1428571428571425E-2</v>
       </c>
       <c r="G2" s="5">
         <f t="shared" si="0"/>
-        <v>7.6923076923076927E-2</v>
+        <v>7.1428571428571425E-2</v>
       </c>
       <c r="H2" s="5">
         <f t="shared" si="0"/>
-        <v>7.6923076923076927E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>7.1428571428571425E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3">
-        <v>0.09</v>
-      </c>
-      <c r="C3">
-        <v>0.09</v>
-      </c>
-      <c r="D3">
-        <v>0.09</v>
-      </c>
-      <c r="E3">
-        <v>0.09</v>
-      </c>
-      <c r="F3">
-        <v>0.09</v>
-      </c>
-      <c r="G3">
-        <v>0.09</v>
-      </c>
-      <c r="H3">
-        <v>0.09</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="5">
+        <f>1/23</f>
+        <v>4.3478260869565216E-2</v>
+      </c>
+      <c r="C3" s="5">
+        <f t="shared" ref="C3:H3" si="1">1/23</f>
+        <v>4.3478260869565216E-2</v>
+      </c>
+      <c r="D3" s="5">
+        <f t="shared" si="1"/>
+        <v>4.3478260869565216E-2</v>
+      </c>
+      <c r="E3" s="5">
+        <f t="shared" si="1"/>
+        <v>4.3478260869565216E-2</v>
+      </c>
+      <c r="F3" s="5">
+        <f t="shared" si="1"/>
+        <v>4.3478260869565216E-2</v>
+      </c>
+      <c r="G3" s="5">
+        <f t="shared" si="1"/>
+        <v>4.3478260869565216E-2</v>
+      </c>
+      <c r="H3" s="5">
+        <f t="shared" si="1"/>
+        <v>4.3478260869565216E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -663,7 +670,7 @@
         <v>4.1599999999999998E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -689,56 +696,70 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
-      <c r="B6">
-        <v>2.9819999999999999E-2</v>
-      </c>
-      <c r="C6">
-        <v>2.9819999999999999E-2</v>
-      </c>
-      <c r="D6">
-        <v>2.9819999999999999E-2</v>
-      </c>
-      <c r="E6">
-        <v>2.9819999999999999E-2</v>
-      </c>
-      <c r="F6">
-        <v>2.9819999999999999E-2</v>
-      </c>
-      <c r="G6">
-        <v>2.9819999999999999E-2</v>
-      </c>
-      <c r="H6">
-        <v>2.9819999999999999E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="5">
+        <f>1/33</f>
+        <v>3.0303030303030304E-2</v>
+      </c>
+      <c r="C6" s="5">
+        <f t="shared" ref="C6:H6" si="2">1/33</f>
+        <v>3.0303030303030304E-2</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="2"/>
+        <v>3.0303030303030304E-2</v>
+      </c>
+      <c r="E6" s="5">
+        <f t="shared" si="2"/>
+        <v>3.0303030303030304E-2</v>
+      </c>
+      <c r="F6" s="5">
+        <f t="shared" si="2"/>
+        <v>3.0303030303030304E-2</v>
+      </c>
+      <c r="G6" s="5">
+        <f t="shared" si="2"/>
+        <v>3.0303030303030304E-2</v>
+      </c>
+      <c r="H6" s="5">
+        <f t="shared" si="2"/>
+        <v>3.0303030303030304E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>17</v>
       </c>
-      <c r="B7">
-        <v>5.8700000000000002E-2</v>
-      </c>
-      <c r="C7">
-        <v>5.8700000000000002E-2</v>
-      </c>
-      <c r="D7">
-        <v>6.8000000000000005E-2</v>
-      </c>
-      <c r="E7">
-        <v>5.8700000000000002E-2</v>
-      </c>
-      <c r="F7">
-        <v>5.8700000000000002E-2</v>
-      </c>
-      <c r="G7">
-        <v>5.8700000000000002E-2</v>
-      </c>
-      <c r="H7">
-        <v>5.8700000000000002E-2</v>
+      <c r="B7" s="5">
+        <f>1/17</f>
+        <v>5.8823529411764705E-2</v>
+      </c>
+      <c r="C7" s="5">
+        <f t="shared" ref="C7:H7" si="3">1/17</f>
+        <v>5.8823529411764705E-2</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="3"/>
+        <v>5.8823529411764705E-2</v>
+      </c>
+      <c r="E7" s="5">
+        <f t="shared" si="3"/>
+        <v>5.8823529411764705E-2</v>
+      </c>
+      <c r="F7" s="5">
+        <f t="shared" si="3"/>
+        <v>5.8823529411764705E-2</v>
+      </c>
+      <c r="G7" s="5">
+        <f t="shared" si="3"/>
+        <v>5.8823529411764705E-2</v>
+      </c>
+      <c r="H7" s="5">
+        <f t="shared" si="3"/>
+        <v>5.8823529411764705E-2</v>
       </c>
     </row>
   </sheetData>
@@ -752,13 +773,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:H7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
-    <col min="2" max="8" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="19.1796875" customWidth="1"/>
+    <col min="2" max="8" width="14.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="4" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>18</v>
       </c>
@@ -784,59 +805,73 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="C2">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="D2">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="E2">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="F2">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="G2">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="H2">
-        <v>7.1999999999999995E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="5">
+        <f>1/14</f>
+        <v>7.1428571428571425E-2</v>
+      </c>
+      <c r="C2" s="5">
+        <f t="shared" ref="C2:H2" si="0">1/14</f>
+        <v>7.1428571428571425E-2</v>
+      </c>
+      <c r="D2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.1428571428571425E-2</v>
+      </c>
+      <c r="E2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.1428571428571425E-2</v>
+      </c>
+      <c r="F2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.1428571428571425E-2</v>
+      </c>
+      <c r="G2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.1428571428571425E-2</v>
+      </c>
+      <c r="H2" s="5">
+        <f t="shared" si="0"/>
+        <v>7.1428571428571425E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-      <c r="C3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-      <c r="D3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-      <c r="E3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-      <c r="F3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-      <c r="G3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-      <c r="H3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="5">
+        <f>1/28</f>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="C3" s="5">
+        <f t="shared" ref="C3:H3" si="1">1/28</f>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="D3" s="5">
+        <f t="shared" si="1"/>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="E3" s="5">
+        <f t="shared" si="1"/>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="F3" s="5">
+        <f t="shared" si="1"/>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="G3" s="5">
+        <f t="shared" si="1"/>
+        <v>3.5714285714285712E-2</v>
+      </c>
+      <c r="H3" s="5">
+        <f t="shared" si="1"/>
+        <v>3.5714285714285712E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -862,7 +897,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -888,7 +923,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -914,7 +949,7 @@
         <v>3.0300000000000001E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>17</v>
       </c>

</xml_diff>